<commit_message>
Bottom LCSC BOM updated
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Top Board/_BOM/SM_Top_PCB_LCSC.xlsx
+++ b/Deliverables/SM_Top Board/_BOM/SM_Top_PCB_LCSC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\ColeBenson-SmartMotors\Deliverables\SM_Top Board\_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A4D011A-C39B-492F-909C-166B54BCC6EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4060B9E-6605-424E-A422-D3FAD764FA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -729,9 +729,6 @@
     <t>Texas Instruments</t>
   </si>
   <si>
-    <t>Farnell</t>
-  </si>
-  <si>
     <t>DIODES INC.</t>
   </si>
   <si>
@@ -994,6 +991,9 @@
   </si>
   <si>
     <t>Unable to find chinese supplier. Farnell has 11 parts in stock</t>
+  </si>
+  <si>
+    <t>Local Supplier</t>
   </si>
 </sst>
 </file>
@@ -1303,7 +1303,16 @@
     </xf>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="5" xfId="2" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1315,7 +1324,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1325,15 +1334,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1640,27 +1640,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
-      <c r="M1" s="30"/>
-      <c r="N1" s="30"/>
-      <c r="O1" s="30"/>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="30"/>
-      <c r="R1" s="30"/>
-      <c r="S1" s="31"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
+      <c r="L1" s="33"/>
+      <c r="M1" s="33"/>
+      <c r="N1" s="33"/>
+      <c r="O1" s="33"/>
+      <c r="P1" s="33"/>
+      <c r="Q1" s="33"/>
+      <c r="R1" s="33"/>
+      <c r="S1" s="34"/>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
@@ -1685,7 +1685,7 @@
         <v>210</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="I2" s="6" t="s">
         <v>211</v>
@@ -1694,7 +1694,7 @@
         <v>212</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="L2" s="6" t="s">
         <v>213</v>
@@ -1718,14 +1718,14 @@
         <v>219</v>
       </c>
       <c r="S2" s="6" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A3" s="8">
         <v>1</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="35" t="s">
         <v>220</v>
       </c>
       <c r="C3" s="9" t="s">
@@ -1741,10 +1741,10 @@
         <v>6</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="I3" s="20"/>
       <c r="J3" s="9" t="s">
@@ -1761,7 +1761,7 @@
         <v>10</v>
       </c>
       <c r="N3" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O3" s="11">
         <v>0.24909999999999999</v>
@@ -1784,7 +1784,7 @@
         <f>A3+1</f>
         <v>2</v>
       </c>
-      <c r="B4" s="28"/>
+      <c r="B4" s="35"/>
       <c r="C4" s="9" t="s">
         <v>8</v>
       </c>
@@ -1798,10 +1798,10 @@
         <v>11</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="I4" s="21"/>
       <c r="J4" s="9" t="s">
@@ -1818,7 +1818,7 @@
         <v>40</v>
       </c>
       <c r="N4" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O4" s="11">
         <v>4.0000000000000001E-3</v>
@@ -1841,7 +1841,7 @@
         <f t="shared" ref="A5:A56" si="1">A4+1</f>
         <v>3</v>
       </c>
-      <c r="B5" s="28"/>
+      <c r="B5" s="35"/>
       <c r="C5" s="9" t="s">
         <v>13</v>
       </c>
@@ -1855,13 +1855,13 @@
         <v>16</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="H5" s="9" t="s">
+        <v>268</v>
+      </c>
+      <c r="I5" s="21" t="s">
         <v>269</v>
-      </c>
-      <c r="I5" s="21" t="s">
-        <v>270</v>
       </c>
       <c r="J5" s="9" t="s">
         <v>12</v>
@@ -1877,7 +1877,7 @@
         <v>5</v>
       </c>
       <c r="N5" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O5" s="11">
         <v>9.8400000000000001E-2</v>
@@ -1894,7 +1894,7 @@
         <v>0.49199999999999999</v>
       </c>
       <c r="S5" s="5" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6" spans="1:19" ht="38.25" x14ac:dyDescent="0.25">
@@ -1902,7 +1902,7 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="B6" s="28"/>
+      <c r="B6" s="35"/>
       <c r="C6" s="9" t="s">
         <v>18</v>
       </c>
@@ -1916,10 +1916,10 @@
         <v>20</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="I6" s="20"/>
       <c r="J6" s="9" t="s">
@@ -1936,7 +1936,7 @@
         <v>5</v>
       </c>
       <c r="N6" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O6" s="11">
         <v>0.4869</v>
@@ -1949,7 +1949,7 @@
         <v>0.4869</v>
       </c>
       <c r="R6" s="12">
-        <f t="shared" ref="R6:R55" si="2">Q6*M6</f>
+        <f t="shared" ref="R6:R54" si="2">Q6*M6</f>
         <v>2.4344999999999999</v>
       </c>
       <c r="S6" s="5"/>
@@ -1959,7 +1959,7 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="B7" s="28"/>
+      <c r="B7" s="35"/>
       <c r="C7" s="9" t="s">
         <v>22</v>
       </c>
@@ -1973,10 +1973,10 @@
         <v>24</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I7" s="20"/>
       <c r="J7" s="9" t="s">
@@ -1993,7 +1993,7 @@
         <v>5</v>
       </c>
       <c r="N7" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O7" s="11">
         <v>7.1099999999999997E-2</v>
@@ -2016,7 +2016,7 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="B8" s="28"/>
+      <c r="B8" s="35"/>
       <c r="C8" s="9" t="s">
         <v>26</v>
       </c>
@@ -2033,7 +2033,7 @@
         <v>230</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="I8" s="20"/>
       <c r="J8" s="9" t="s">
@@ -2050,7 +2050,7 @@
         <v>5</v>
       </c>
       <c r="N8" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O8" s="11">
         <v>5.3E-3</v>
@@ -2073,7 +2073,7 @@
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="B9" s="28"/>
+      <c r="B9" s="35"/>
       <c r="C9" s="9" t="s">
         <v>30</v>
       </c>
@@ -2087,10 +2087,10 @@
         <v>33</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="I9" s="21"/>
       <c r="J9" s="9" t="s">
@@ -2107,7 +2107,7 @@
         <v>5</v>
       </c>
       <c r="N9" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O9" s="11">
         <v>3.27E-2</v>
@@ -2130,7 +2130,7 @@
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="B10" s="28"/>
+      <c r="B10" s="35"/>
       <c r="C10" s="9" t="s">
         <v>35</v>
       </c>
@@ -2144,10 +2144,10 @@
         <v>37</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="I10" s="21"/>
       <c r="J10" s="9" t="s">
@@ -2164,7 +2164,7 @@
         <v>5</v>
       </c>
       <c r="N10" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O10" s="11">
         <v>0.30170000000000002</v>
@@ -2187,7 +2187,7 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="B11" s="28"/>
+      <c r="B11" s="35"/>
       <c r="C11" s="9" t="s">
         <v>38</v>
       </c>
@@ -2204,7 +2204,7 @@
         <v>230</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="I11" s="20"/>
       <c r="J11" s="9" t="s">
@@ -2221,13 +2221,13 @@
         <v>5</v>
       </c>
       <c r="N11" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O11" s="11">
         <v>1.2200000000000001E-2</v>
       </c>
       <c r="P11" s="12">
-        <f>O11*K11</f>
+        <f t="shared" ref="P11:P16" si="4">O11*K11</f>
         <v>0.61</v>
       </c>
       <c r="Q11" s="11">
@@ -2244,7 +2244,7 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="B12" s="28"/>
+      <c r="B12" s="35"/>
       <c r="C12" s="9" t="s">
         <v>42</v>
       </c>
@@ -2258,10 +2258,10 @@
         <v>44</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="I12" s="21"/>
       <c r="J12" s="9" t="s">
@@ -2278,13 +2278,13 @@
         <v>25</v>
       </c>
       <c r="N12" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O12" s="11">
         <v>3.9300000000000002E-2</v>
       </c>
       <c r="P12" s="12">
-        <f>O12*K12</f>
+        <f t="shared" si="4"/>
         <v>0.39300000000000002</v>
       </c>
       <c r="Q12" s="11">
@@ -2301,7 +2301,7 @@
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
-      <c r="B13" s="28"/>
+      <c r="B13" s="35"/>
       <c r="C13" s="9" t="s">
         <v>46</v>
       </c>
@@ -2315,10 +2315,10 @@
         <v>48</v>
       </c>
       <c r="G13" s="9" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="H13" s="9" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="I13" s="21"/>
       <c r="J13" s="9" t="s">
@@ -2335,13 +2335,13 @@
         <v>10</v>
       </c>
       <c r="N13" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O13" s="11">
         <v>2.5899999999999999E-2</v>
       </c>
       <c r="P13" s="12">
-        <f>O13*K13</f>
+        <f t="shared" si="4"/>
         <v>0.51800000000000002</v>
       </c>
       <c r="Q13" s="11">
@@ -2358,7 +2358,7 @@
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="B14" s="28"/>
+      <c r="B14" s="35"/>
       <c r="C14" s="9" t="s">
         <v>49</v>
       </c>
@@ -2372,10 +2372,10 @@
         <v>51</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="I14" s="22"/>
       <c r="J14" s="9" t="s">
@@ -2392,13 +2392,13 @@
         <v>10</v>
       </c>
       <c r="N14" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O14" s="11">
         <v>7.4999999999999997E-3</v>
       </c>
       <c r="P14" s="12">
-        <f>O14*K14</f>
+        <f t="shared" si="4"/>
         <v>0.375</v>
       </c>
       <c r="Q14" s="11">
@@ -2415,27 +2415,27 @@
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
-      <c r="B15" s="28"/>
+      <c r="B15" s="35"/>
       <c r="C15" s="9" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>15</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="H15" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="I15" s="2" t="s">
         <v>283</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>284</v>
       </c>
       <c r="J15" s="9" t="s">
         <v>52</v>
@@ -2451,13 +2451,13 @@
         <v>20</v>
       </c>
       <c r="N15" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O15" s="11">
         <v>1.9300000000000001E-2</v>
       </c>
       <c r="P15" s="12">
-        <f>O15*K15</f>
+        <f t="shared" si="4"/>
         <v>0.38600000000000001</v>
       </c>
       <c r="Q15" s="11">
@@ -2474,24 +2474,24 @@
         <f>A15+1</f>
         <v>14</v>
       </c>
-      <c r="B16" s="28"/>
+      <c r="B16" s="35"/>
       <c r="C16" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="E16" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="F16" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="F16" s="2" t="s">
-        <v>260</v>
-      </c>
       <c r="G16" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="I16" s="23"/>
       <c r="J16" s="2" t="s">
@@ -2508,13 +2508,13 @@
         <v>20</v>
       </c>
       <c r="N16" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O16" s="4">
         <v>4.9399999999999999E-2</v>
       </c>
       <c r="P16" s="12">
-        <f>O16*K16</f>
+        <f t="shared" si="4"/>
         <v>0.49399999999999999</v>
       </c>
       <c r="Q16" s="4">
@@ -2531,7 +2531,7 @@
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="B17" s="28"/>
+      <c r="B17" s="35"/>
       <c r="C17" s="9" t="s">
         <v>54</v>
       </c>
@@ -2545,10 +2545,10 @@
         <v>56</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="I17" s="20"/>
       <c r="J17" s="9" t="s">
@@ -2565,7 +2565,7 @@
         <v>5</v>
       </c>
       <c r="N17" s="15" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="O17" s="11">
         <v>0.1</v>
@@ -2588,7 +2588,7 @@
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
-      <c r="B18" s="28"/>
+      <c r="B18" s="35"/>
       <c r="C18" s="9" t="s">
         <v>30</v>
       </c>
@@ -2602,10 +2602,10 @@
         <v>33</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="I18" s="20"/>
       <c r="J18" s="9" t="s">
@@ -2622,7 +2622,7 @@
         <v>5</v>
       </c>
       <c r="N18" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O18" s="11">
         <v>3.27E-2</v>
@@ -2631,7 +2631,7 @@
         <f>O18*K18</f>
         <v>0.65400000000000003</v>
       </c>
-      <c r="Q18" s="38">
+      <c r="Q18" s="31">
         <v>3.27E-2</v>
       </c>
       <c r="R18" s="12">
@@ -2645,7 +2645,7 @@
         <f t="shared" si="1"/>
         <v>17</v>
       </c>
-      <c r="B19" s="33" t="s">
+      <c r="B19" s="36" t="s">
         <v>221</v>
       </c>
       <c r="C19" s="9" t="s">
@@ -2661,10 +2661,10 @@
         <v>63</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="I19" s="22"/>
       <c r="J19" s="9" t="s">
@@ -2681,7 +2681,7 @@
         <v>20</v>
       </c>
       <c r="N19" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O19" s="11">
         <v>4.7000000000000002E-3</v>
@@ -2704,7 +2704,7 @@
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
-      <c r="B20" s="34"/>
+      <c r="B20" s="37"/>
       <c r="C20" s="9" t="s">
         <v>65</v>
       </c>
@@ -2718,10 +2718,10 @@
         <v>64</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="I20" s="22"/>
       <c r="J20" s="9" t="s">
@@ -2738,7 +2738,7 @@
         <v>5</v>
       </c>
       <c r="N20" s="15" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="O20" s="4">
         <v>0.66</v>
@@ -2761,7 +2761,7 @@
         <f t="shared" si="1"/>
         <v>19</v>
       </c>
-      <c r="B21" s="34"/>
+      <c r="B21" s="37"/>
       <c r="C21" s="9" t="s">
         <v>68</v>
       </c>
@@ -2775,7 +2775,7 @@
         <v>67</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="H21" s="9"/>
       <c r="I21" s="22"/>
@@ -2793,7 +2793,7 @@
         <v>40</v>
       </c>
       <c r="N21" s="15" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="O21" s="4">
         <v>0.36</v>
@@ -2816,7 +2816,7 @@
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="B22" s="34"/>
+      <c r="B22" s="37"/>
       <c r="C22" s="9" t="s">
         <v>90</v>
       </c>
@@ -2830,10 +2830,10 @@
         <v>89</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="I22" s="22"/>
       <c r="J22" s="9" t="s">
@@ -2850,7 +2850,7 @@
         <v>5</v>
       </c>
       <c r="N22" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O22" s="11">
         <v>0.14299999999999999</v>
@@ -2873,7 +2873,7 @@
         <f t="shared" si="1"/>
         <v>21</v>
       </c>
-      <c r="B23" s="35"/>
+      <c r="B23" s="38"/>
       <c r="C23" s="9" t="s">
         <v>93</v>
       </c>
@@ -2887,13 +2887,13 @@
         <v>92</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="H23" s="9" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="I23" s="9" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="J23" s="9" t="s">
         <v>92</v>
@@ -2909,7 +2909,7 @@
         <v>5</v>
       </c>
       <c r="N23" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O23" s="4">
         <v>7.5800000000000006E-2</v>
@@ -2926,7 +2926,7 @@
         <v>0.75800000000000001</v>
       </c>
       <c r="S23" s="13" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
@@ -2950,10 +2950,10 @@
         <v>71</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="I24" s="9"/>
       <c r="J24" s="9" t="s">
@@ -2970,7 +2970,7 @@
         <v>5</v>
       </c>
       <c r="N24" s="15" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="O24" s="4">
         <v>0.14899999999999999</v>
@@ -3009,10 +3009,10 @@
         <v>86</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="I25" s="9"/>
       <c r="J25" s="9" t="s">
@@ -3029,7 +3029,7 @@
         <v>5</v>
       </c>
       <c r="N25" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O25" s="4">
         <v>0.79710000000000003</v>
@@ -3068,10 +3068,10 @@
         <v>108</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="I26" s="9"/>
       <c r="J26" s="9" t="s">
@@ -3088,7 +3088,7 @@
         <v>40</v>
       </c>
       <c r="N26" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O26" s="4">
         <v>2.4777</v>
@@ -3111,7 +3111,7 @@
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="B27" s="33" t="s">
+      <c r="B27" s="36" t="s">
         <v>225</v>
       </c>
       <c r="C27" s="9" t="s">
@@ -3127,10 +3127,10 @@
         <v>115</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I27" s="9"/>
       <c r="J27" s="9" t="s">
@@ -3147,7 +3147,7 @@
         <v>10</v>
       </c>
       <c r="N27" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O27" s="4">
         <v>1.6999999999999999E-3</v>
@@ -3170,7 +3170,7 @@
         <f t="shared" si="1"/>
         <v>26</v>
       </c>
-      <c r="B28" s="34"/>
+      <c r="B28" s="37"/>
       <c r="C28" s="9" t="s">
         <v>117</v>
       </c>
@@ -3187,7 +3187,7 @@
         <v>230</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="I28" s="9"/>
       <c r="J28" s="9" t="s">
@@ -3204,7 +3204,7 @@
         <v>10</v>
       </c>
       <c r="N28" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O28" s="4">
         <v>1.6999999999999999E-3</v>
@@ -3227,7 +3227,7 @@
         <f t="shared" si="1"/>
         <v>27</v>
       </c>
-      <c r="B29" s="34"/>
+      <c r="B29" s="37"/>
       <c r="C29" s="9" t="s">
         <v>121</v>
       </c>
@@ -3244,7 +3244,7 @@
         <v>230</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="I29" s="9"/>
       <c r="J29" s="9" t="s">
@@ -3261,7 +3261,7 @@
         <v>5</v>
       </c>
       <c r="N29" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O29" s="4">
         <v>2.0999999999999999E-3</v>
@@ -3284,7 +3284,7 @@
         <f t="shared" si="1"/>
         <v>28</v>
       </c>
-      <c r="B30" s="34"/>
+      <c r="B30" s="37"/>
       <c r="C30" s="9" t="s">
         <v>125</v>
       </c>
@@ -3301,7 +3301,7 @@
         <v>230</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="I30" s="9"/>
       <c r="J30" s="9" t="s">
@@ -3318,20 +3318,20 @@
         <v>5</v>
       </c>
       <c r="N30" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O30" s="11">
         <v>1.4E-3</v>
       </c>
       <c r="P30" s="12">
-        <f t="shared" ref="P30:P32" si="4">O30*K30</f>
+        <f t="shared" ref="P30:P31" si="5">O30*K30</f>
         <v>0.13999999999999999</v>
       </c>
       <c r="Q30" s="11">
         <v>1.4E-3</v>
       </c>
       <c r="R30" s="12">
-        <f t="shared" ref="R30:R32" si="5">Q30*K30</f>
+        <f t="shared" ref="R30:R31" si="6">Q30*K30</f>
         <v>0.13999999999999999</v>
       </c>
       <c r="S30" s="5"/>
@@ -3341,7 +3341,7 @@
         <f t="shared" si="1"/>
         <v>29</v>
       </c>
-      <c r="B31" s="34"/>
+      <c r="B31" s="37"/>
       <c r="C31" s="9" t="s">
         <v>129</v>
       </c>
@@ -3358,7 +3358,7 @@
         <v>230</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="I31" s="5"/>
       <c r="J31" s="9" t="s">
@@ -3375,20 +3375,20 @@
         <v>20</v>
       </c>
       <c r="N31" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O31" s="11">
         <v>2.3E-3</v>
       </c>
       <c r="P31" s="12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.22999999999999998</v>
       </c>
       <c r="Q31" s="11">
         <v>2.3E-3</v>
       </c>
       <c r="R31" s="12">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.22999999999999998</v>
       </c>
       <c r="S31" s="5"/>
@@ -3398,7 +3398,7 @@
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
-      <c r="B32" s="34"/>
+      <c r="B32" s="37"/>
       <c r="C32" s="9" t="s">
         <v>133</v>
       </c>
@@ -3414,8 +3414,8 @@
       <c r="G32" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="H32" s="36" t="s">
-        <v>301</v>
+      <c r="H32" s="29" t="s">
+        <v>300</v>
       </c>
       <c r="I32" s="5"/>
       <c r="J32" s="9" t="s">
@@ -3431,14 +3431,14 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="N32" s="37" t="s">
-        <v>263</v>
+      <c r="N32" s="30" t="s">
+        <v>262</v>
       </c>
       <c r="O32" s="11">
         <v>8.5699999999999998E-2</v>
       </c>
       <c r="P32" s="12">
-        <f>O32*K32</f>
+        <f t="shared" ref="P32:P40" si="7">O32*K32</f>
         <v>0.42849999999999999</v>
       </c>
       <c r="Q32" s="11">
@@ -3455,7 +3455,7 @@
         <f t="shared" si="1"/>
         <v>31</v>
       </c>
-      <c r="B33" s="34"/>
+      <c r="B33" s="37"/>
       <c r="C33" s="9" t="s">
         <v>138</v>
       </c>
@@ -3472,7 +3472,7 @@
         <v>230</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I33" s="5"/>
       <c r="J33" s="9" t="s">
@@ -3489,20 +3489,20 @@
         <v>40</v>
       </c>
       <c r="N33" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O33" s="11">
         <v>2.2000000000000001E-3</v>
       </c>
       <c r="P33" s="12">
-        <f>O33*K33</f>
+        <f t="shared" si="7"/>
         <v>0.22</v>
       </c>
       <c r="Q33" s="11">
         <v>2.2000000000000001E-3</v>
       </c>
       <c r="R33" s="12">
-        <f>Q33*K33</f>
+        <f t="shared" ref="R33:R40" si="8">Q33*K33</f>
         <v>0.22</v>
       </c>
       <c r="S33" s="5"/>
@@ -3512,7 +3512,7 @@
         <f t="shared" si="1"/>
         <v>32</v>
       </c>
-      <c r="B34" s="34"/>
+      <c r="B34" s="37"/>
       <c r="C34" s="9" t="s">
         <v>142</v>
       </c>
@@ -3529,7 +3529,7 @@
         <v>231</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="I34" s="5"/>
       <c r="J34" s="9" t="s">
@@ -3546,20 +3546,20 @@
         <v>5</v>
       </c>
       <c r="N34" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O34" s="11">
         <v>9.2999999999999992E-3</v>
       </c>
       <c r="P34" s="12">
-        <f>O34*K34</f>
+        <f t="shared" si="7"/>
         <v>0.46499999999999997</v>
       </c>
       <c r="Q34" s="11">
         <v>9.2999999999999992E-3</v>
       </c>
       <c r="R34" s="12">
-        <f>Q34*K34</f>
+        <f t="shared" si="8"/>
         <v>0.46499999999999997</v>
       </c>
       <c r="S34" s="5"/>
@@ -3569,7 +3569,7 @@
         <f t="shared" si="1"/>
         <v>33</v>
       </c>
-      <c r="B35" s="34"/>
+      <c r="B35" s="37"/>
       <c r="C35" s="9" t="s">
         <v>146</v>
       </c>
@@ -3586,7 +3586,7 @@
         <v>230</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="I35" s="5"/>
       <c r="J35" s="9" t="s">
@@ -3603,20 +3603,20 @@
         <v>5</v>
       </c>
       <c r="N35" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O35" s="11">
         <v>2E-3</v>
       </c>
       <c r="P35" s="12">
-        <f>O35*K35</f>
+        <f t="shared" si="7"/>
         <v>0.2</v>
       </c>
       <c r="Q35" s="11">
         <v>2E-3</v>
       </c>
       <c r="R35" s="12">
-        <f>Q35*K35</f>
+        <f t="shared" si="8"/>
         <v>0.2</v>
       </c>
       <c r="S35" s="5"/>
@@ -3626,7 +3626,7 @@
         <f t="shared" si="1"/>
         <v>34</v>
       </c>
-      <c r="B36" s="34"/>
+      <c r="B36" s="37"/>
       <c r="C36" s="9" t="s">
         <v>150</v>
       </c>
@@ -3643,7 +3643,7 @@
         <v>231</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="I36" s="5"/>
       <c r="J36" s="9" t="s">
@@ -3660,20 +3660,20 @@
         <v>5</v>
       </c>
       <c r="N36" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O36" s="11">
         <v>5.7999999999999996E-3</v>
       </c>
       <c r="P36" s="12">
-        <f>O36*K36</f>
+        <f t="shared" si="7"/>
         <v>0.28999999999999998</v>
       </c>
       <c r="Q36" s="11">
         <v>5.7999999999999996E-3</v>
       </c>
       <c r="R36" s="12">
-        <f>Q36*K36</f>
+        <f t="shared" si="8"/>
         <v>0.28999999999999998</v>
       </c>
       <c r="S36" s="5"/>
@@ -3683,7 +3683,7 @@
         <f t="shared" si="1"/>
         <v>35</v>
       </c>
-      <c r="B37" s="34"/>
+      <c r="B37" s="37"/>
       <c r="C37" s="9" t="s">
         <v>154</v>
       </c>
@@ -3700,7 +3700,7 @@
         <v>230</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="I37" s="5"/>
       <c r="J37" s="9" t="s">
@@ -3717,20 +3717,20 @@
         <v>5</v>
       </c>
       <c r="N37" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O37" s="11">
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="P37" s="12">
-        <f>O37*K37</f>
+        <f t="shared" si="7"/>
         <v>0.21</v>
       </c>
       <c r="Q37" s="11">
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="R37" s="12">
-        <f>Q37*K37</f>
+        <f t="shared" si="8"/>
         <v>0.21</v>
       </c>
       <c r="S37" s="5"/>
@@ -3740,7 +3740,7 @@
         <f t="shared" si="1"/>
         <v>36</v>
       </c>
-      <c r="B38" s="34"/>
+      <c r="B38" s="37"/>
       <c r="C38" s="9" t="s">
         <v>158</v>
       </c>
@@ -3757,7 +3757,7 @@
         <v>231</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="I38" s="5"/>
       <c r="J38" s="9" t="s">
@@ -3774,20 +3774,20 @@
         <v>5</v>
       </c>
       <c r="N38" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O38" s="11">
         <v>9.2999999999999992E-3</v>
       </c>
       <c r="P38" s="12">
-        <f>O38*K38</f>
+        <f t="shared" si="7"/>
         <v>0.92999999999999994</v>
       </c>
       <c r="Q38" s="11">
         <v>9.2999999999999992E-3</v>
       </c>
       <c r="R38" s="12">
-        <f>Q38*K38</f>
+        <f t="shared" si="8"/>
         <v>0.92999999999999994</v>
       </c>
       <c r="S38" s="5"/>
@@ -3797,7 +3797,7 @@
         <f t="shared" si="1"/>
         <v>37</v>
       </c>
-      <c r="B39" s="34"/>
+      <c r="B39" s="37"/>
       <c r="C39" s="9" t="s">
         <v>162</v>
       </c>
@@ -3814,7 +3814,7 @@
         <v>230</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="I39" s="5"/>
       <c r="J39" s="9" t="s">
@@ -3831,20 +3831,20 @@
         <v>5</v>
       </c>
       <c r="N39" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O39" s="11">
         <v>2.5999999999999999E-3</v>
       </c>
       <c r="P39" s="12">
-        <f>O39*K39</f>
+        <f t="shared" si="7"/>
         <v>0.26</v>
       </c>
       <c r="Q39" s="11">
         <v>2.5999999999999999E-3</v>
       </c>
       <c r="R39" s="12">
-        <f>Q39*K39</f>
+        <f t="shared" si="8"/>
         <v>0.26</v>
       </c>
       <c r="S39" s="5"/>
@@ -3854,7 +3854,7 @@
         <f t="shared" si="1"/>
         <v>38</v>
       </c>
-      <c r="B40" s="35"/>
+      <c r="B40" s="38"/>
       <c r="C40" s="9" t="s">
         <v>166</v>
       </c>
@@ -3871,7 +3871,7 @@
         <v>230</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="I40" s="5"/>
       <c r="J40" s="9" t="s">
@@ -3888,20 +3888,20 @@
         <v>5</v>
       </c>
       <c r="N40" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O40" s="11">
         <v>2E-3</v>
       </c>
       <c r="P40" s="12">
-        <f>O40*K40</f>
+        <f t="shared" si="7"/>
         <v>0.2</v>
       </c>
       <c r="Q40" s="11">
         <v>2E-3</v>
       </c>
       <c r="R40" s="12">
-        <f>Q40*K40</f>
+        <f t="shared" si="8"/>
         <v>0.2</v>
       </c>
       <c r="S40" s="5"/>
@@ -3911,7 +3911,7 @@
         <f t="shared" si="1"/>
         <v>39</v>
       </c>
-      <c r="B41" s="33" t="s">
+      <c r="B41" s="36" t="s">
         <v>226</v>
       </c>
       <c r="C41" s="9" t="s">
@@ -3965,7 +3965,7 @@
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="B42" s="35"/>
+      <c r="B42" s="38"/>
       <c r="C42" s="9" t="s">
         <v>176</v>
       </c>
@@ -3979,10 +3979,10 @@
         <v>175</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="H42" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="I42" s="5"/>
       <c r="J42" s="9" t="s">
@@ -3999,7 +3999,7 @@
         <v>10</v>
       </c>
       <c r="N42" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O42" s="11">
         <v>0.28860000000000002</v>
@@ -4022,7 +4022,7 @@
         <f t="shared" si="1"/>
         <v>41</v>
       </c>
-      <c r="B43" s="33" t="s">
+      <c r="B43" s="36" t="s">
         <v>227</v>
       </c>
       <c r="C43" s="9" t="s">
@@ -4041,7 +4041,7 @@
         <v>233</v>
       </c>
       <c r="H43" s="5" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="I43" s="5"/>
       <c r="J43" s="9" t="s">
@@ -4058,7 +4058,7 @@
         <v>5</v>
       </c>
       <c r="N43" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O43" s="11">
         <v>0.18729999999999999</v>
@@ -4080,7 +4080,7 @@
         <f t="shared" si="1"/>
         <v>42</v>
       </c>
-      <c r="B44" s="34"/>
+      <c r="B44" s="37"/>
       <c r="C44" s="9" t="s">
         <v>183</v>
       </c>
@@ -4094,10 +4094,10 @@
         <v>182</v>
       </c>
       <c r="G44" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="H44" s="5" t="s">
         <v>313</v>
-      </c>
-      <c r="H44" s="5" t="s">
-        <v>314</v>
       </c>
       <c r="I44" s="5"/>
       <c r="J44" s="9" t="s">
@@ -4114,7 +4114,7 @@
         <v>5</v>
       </c>
       <c r="N44" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O44" s="11">
         <v>0.3478</v>
@@ -4137,7 +4137,7 @@
         <f t="shared" si="1"/>
         <v>43</v>
       </c>
-      <c r="B45" s="34"/>
+      <c r="B45" s="37"/>
       <c r="C45" s="9" t="s">
         <v>187</v>
       </c>
@@ -4154,7 +4154,7 @@
         <v>233</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="I45" s="5"/>
       <c r="J45" s="9" t="s">
@@ -4171,7 +4171,7 @@
         <v>5</v>
       </c>
       <c r="N45" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O45" s="11">
         <v>1.5923</v>
@@ -4194,7 +4194,7 @@
         <f t="shared" si="1"/>
         <v>44</v>
       </c>
-      <c r="B46" s="34"/>
+      <c r="B46" s="37"/>
       <c r="C46" s="9" t="s">
         <v>191</v>
       </c>
@@ -4208,7 +4208,7 @@
         <v>190</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H46" s="5"/>
       <c r="I46" s="5"/>
@@ -4226,7 +4226,7 @@
         <v>5</v>
       </c>
       <c r="N46" s="15" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="O46" s="11">
         <v>0.34639999999999999</v>
@@ -4249,7 +4249,7 @@
         <f t="shared" si="1"/>
         <v>45</v>
       </c>
-      <c r="B47" s="34"/>
+      <c r="B47" s="37"/>
       <c r="C47" s="9" t="s">
         <v>195</v>
       </c>
@@ -4263,10 +4263,10 @@
         <v>194</v>
       </c>
       <c r="G47" s="5" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H47" s="5" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="I47" s="5"/>
       <c r="J47" s="9" t="s">
@@ -4283,7 +4283,7 @@
         <v>5</v>
       </c>
       <c r="N47" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O47" s="11">
         <v>0.30620000000000003</v>
@@ -4306,7 +4306,7 @@
         <f t="shared" si="1"/>
         <v>46</v>
       </c>
-      <c r="B48" s="34"/>
+      <c r="B48" s="37"/>
       <c r="C48" s="9" t="s">
         <v>199</v>
       </c>
@@ -4361,7 +4361,7 @@
         <f t="shared" si="1"/>
         <v>47</v>
       </c>
-      <c r="B49" s="35"/>
+      <c r="B49" s="38"/>
       <c r="C49" s="9" t="s">
         <v>203</v>
       </c>
@@ -4375,7 +4375,7 @@
         <v>202</v>
       </c>
       <c r="G49" s="5" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="H49" s="5"/>
       <c r="I49" s="5"/>
@@ -4393,7 +4393,7 @@
         <v>5</v>
       </c>
       <c r="N49" s="15" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="O49" s="11">
         <v>1.92</v>
@@ -4416,7 +4416,7 @@
         <f t="shared" si="1"/>
         <v>48</v>
       </c>
-      <c r="B50" s="32" t="s">
+      <c r="B50" s="28" t="s">
         <v>228</v>
       </c>
       <c r="C50" s="9" t="s">
@@ -4432,10 +4432,10 @@
         <v>74</v>
       </c>
       <c r="G50" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="H50" s="5" t="s">
         <v>317</v>
-      </c>
-      <c r="H50" s="5" t="s">
-        <v>318</v>
       </c>
       <c r="I50" s="5"/>
       <c r="J50" s="9" t="s">
@@ -4452,7 +4452,7 @@
         <v>5</v>
       </c>
       <c r="N50" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O50" s="11">
         <v>1.8448</v>
@@ -4475,7 +4475,7 @@
         <f t="shared" si="1"/>
         <v>49</v>
       </c>
-      <c r="B51" s="32"/>
+      <c r="B51" s="28"/>
       <c r="C51" s="9" t="s">
         <v>78</v>
       </c>
@@ -4489,10 +4489,10 @@
         <v>77</v>
       </c>
       <c r="G51" s="5" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="H51" s="5" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="I51" s="5"/>
       <c r="J51" s="9" t="s">
@@ -4509,7 +4509,7 @@
         <v>10</v>
       </c>
       <c r="N51" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="O51" s="11">
         <v>0.72860000000000003</v>
@@ -4532,7 +4532,7 @@
         <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="B52" s="32"/>
+      <c r="B52" s="28"/>
       <c r="C52" s="9" t="s">
         <v>81</v>
       </c>
@@ -4546,7 +4546,7 @@
         <v>80</v>
       </c>
       <c r="G52" s="5" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="H52" s="5"/>
       <c r="I52" s="5"/>
@@ -4564,24 +4564,24 @@
         <v>5</v>
       </c>
       <c r="N52" s="15" t="s">
-        <v>234</v>
+        <v>322</v>
       </c>
       <c r="O52" s="11">
-        <v>1.27</v>
+        <v>1.74</v>
       </c>
       <c r="P52" s="12">
         <f t="shared" si="3"/>
-        <v>1.27</v>
+        <v>1.74</v>
       </c>
       <c r="Q52" s="11">
-        <v>1.27</v>
+        <v>1.74</v>
       </c>
       <c r="R52" s="12">
         <f t="shared" si="2"/>
-        <v>6.35</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="S52" s="5" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="53" spans="1:19" ht="25.5" x14ac:dyDescent="0.25">
@@ -4589,7 +4589,7 @@
         <f t="shared" si="1"/>
         <v>51</v>
       </c>
-      <c r="B53" s="32"/>
+      <c r="B53" s="28"/>
       <c r="C53" s="9" t="s">
         <v>84</v>
       </c>
@@ -4603,7 +4603,7 @@
         <v>83</v>
       </c>
       <c r="G53" s="5" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="H53" s="5"/>
       <c r="I53" s="5"/>
@@ -4643,7 +4643,7 @@
         <f t="shared" si="1"/>
         <v>52</v>
       </c>
-      <c r="B54" s="32"/>
+      <c r="B54" s="28"/>
       <c r="C54" s="9" t="s">
         <v>97</v>
       </c>
@@ -4657,7 +4657,7 @@
         <v>96</v>
       </c>
       <c r="G54" s="5" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="H54" s="5"/>
       <c r="I54" s="5"/>
@@ -4675,7 +4675,7 @@
         <v>10</v>
       </c>
       <c r="N54" s="15" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="O54" s="11">
         <v>1.61</v>
@@ -4698,7 +4698,7 @@
         <f t="shared" si="1"/>
         <v>53</v>
       </c>
-      <c r="B55" s="32"/>
+      <c r="B55" s="28"/>
       <c r="C55" s="9" t="s">
         <v>104</v>
       </c>
@@ -4712,7 +4712,7 @@
         <v>107</v>
       </c>
       <c r="G55" s="5" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="H55" s="5"/>
       <c r="I55" s="5"/>
@@ -4730,7 +4730,7 @@
         <v>10</v>
       </c>
       <c r="N55" s="15" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="O55" s="11">
         <v>0.19</v>
@@ -4750,7 +4750,7 @@
         <f t="shared" si="1"/>
         <v>54</v>
       </c>
-      <c r="B56" s="32"/>
+      <c r="B56" s="28"/>
       <c r="C56" s="16" t="s">
         <v>100</v>
       </c>
@@ -4780,7 +4780,7 @@
       <c r="N56" s="17"/>
       <c r="O56" s="17"/>
       <c r="P56" s="18">
-        <f t="shared" ref="P56:P57" si="6">O56*L56</f>
+        <f t="shared" ref="P56:P57" si="9">O56*L56</f>
         <v>0</v>
       </c>
       <c r="Q56" s="19"/>
@@ -4822,7 +4822,7 @@
       <c r="N57" s="17"/>
       <c r="O57" s="17"/>
       <c r="P57" s="18">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q57" s="19"/>
@@ -4844,18 +4844,18 @@
       <c r="K58" s="14"/>
       <c r="L58" s="14"/>
       <c r="M58" s="24" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="N58" s="24"/>
       <c r="O58" s="25"/>
       <c r="P58" s="26">
         <f>SUM(P3:P55)</f>
-        <v>73.207199999999986</v>
+        <v>73.677199999999985</v>
       </c>
       <c r="Q58" s="24"/>
       <c r="R58" s="27">
         <f>SUM(R3:R55)</f>
-        <v>245.90749999999994</v>
+        <v>248.25749999999994</v>
       </c>
     </row>
     <row r="59" spans="1:19" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -4961,11 +4961,10 @@
     <hyperlink ref="N55" r:id="rId49" xr:uid="{AABF823B-413E-4EC2-B954-DF074731CAA7}"/>
     <hyperlink ref="N48" r:id="rId50" xr:uid="{1114458F-A78D-4A76-B1CF-305337F52263}"/>
     <hyperlink ref="N53" r:id="rId51" xr:uid="{1E96E8EA-3806-41F4-BDB9-DF5C3FCF6928}"/>
-    <hyperlink ref="N52" r:id="rId52" xr:uid="{9B362694-4504-4DC6-95D1-20D4F3BD5DDD}"/>
-    <hyperlink ref="N41" r:id="rId53" xr:uid="{2F6C76CB-7AFF-4E6D-9732-3183EF2507E8}"/>
+    <hyperlink ref="N41" r:id="rId52" xr:uid="{2F6C76CB-7AFF-4E6D-9732-3183EF2507E8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId54"/>
+  <pageSetup orientation="portrait" r:id="rId53"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>

</xml_diff>